<commit_message>
Sync 249 nonconflicting upstream Bunny Loader sources, UI, localization, font and mod-source features
</commit_message>
<xml_diff>
--- a/docs/referencia/metodos.xlsx
+++ b/docs/referencia/metodos.xlsx
@@ -18158,7 +18158,7 @@
         <x:v>drawParams: tModLoader's BossBarDrawParams (see GlobalBossBar); false removes the game's drawing.</x:v>
       </x:c>
       <x:c r="J483" s="16" t="str">
-        <x:v>BigProgressBarSystem.Draw → BigProgressBarHelper.DrawFancyBar</x:v>
+        <x:v>BigProgressBarSystem.Draw → GUIBossBar.Draw</x:v>
       </x:c>
       <x:c r="K483" s="16" t="str">
         <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModBossBar.js#L33</x:v>
@@ -18193,7 +18193,7 @@
         <x:v>drawParams: tModLoader's BossBarDrawParams (see GlobalBossBar); false removes the game's drawing.</x:v>
       </x:c>
       <x:c r="J484" s="16" t="str">
-        <x:v>BigProgressBarSystem.Draw → BigProgressBarHelper.DrawFancyBar</x:v>
+        <x:v>BigProgressBarSystem.Draw → GUIBossBar.Draw</x:v>
       </x:c>
       <x:c r="K484" s="16" t="str">
         <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModBossBar.js#L32</x:v>

</xml_diff>